<commit_message>
Debug Panel and Mod Update
Applied the Disabled Mods visual at the die/mod icon ownership boundary rather than in disabled_mods_debuff.gd. mod_icon.gd:95 now exposes a small disabled-visual API that applies the existing crossed-out overlay shader to the icon sprite, and dice.gd:821 drives that API from the existing mod disable/enable flow. I also tightened dice.gd:727 so a mod added while the debuff is active is kept suspended and its new icon is immediately marked disabled.
</commit_message>
<xml_diff>
--- a/Docs/pog_names.xlsx
+++ b/Docs/pog_names.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Documents\dicerogue\DiceRogue\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E072F5C5-8F11-4DD9-83B5-6F9C8B7EAF84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01BBABC7-5250-421A-B397-E17E0C34D925}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4180" yWindow="1050" windowWidth="14870" windowHeight="20550" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="380" yWindow="330" windowWidth="31610" windowHeight="20550" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1125,6 +1125,20 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -1153,20 +1167,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1181,7 +1181,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5BDE3407-B5E4-48F0-B629-F7DE39F6B15C}" name="Table1" displayName="Table1" ref="A1:H73" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5BDE3407-B5E4-48F0-B629-F7DE39F6B15C}" name="Table1" displayName="Table1" ref="A1:H73" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
   <autoFilter ref="A1:H73" xr:uid="{5BDE3407-B5E4-48F0-B629-F7DE39F6B15C}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{BC1B2723-41AA-4213-BE45-041E45207073}" name="file"/>

</xml_diff>